<commit_message>
updates shared for 4/9/2026
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\satyam.CLOUDYCOOL\Desktop\Dashboard\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://continuousnet-my.sharepoint.com/personal/satyam_continuous_net/Documents/Desktop/Project Tracker Dashboard/project-dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4665E14-9296-465B-A7EF-B8144438D411}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="13_ncr:1_{C4665E14-9296-465B-A7EF-B8144438D411}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E801EA7F-8186-4A6D-8878-10ED36AC1666}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B5181292-B819-4253-93D6-A2C77ED0862A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="32">
   <si>
     <t xml:space="preserve">Project Name </t>
   </si>
@@ -86,9 +86,6 @@
     <t>Rewst, MS365, HaloPSA, Perimeter81</t>
   </si>
   <si>
-    <t>This project is centered on streamlining the user onboarding process, including updating and optimizing forms and workflows, troubleshooting and resolving workflow issues, and ensuring proper documentation and response management via support tickets.</t>
-  </si>
-  <si>
     <t>Rewst, MS365, Perimeter81, HaloPSA</t>
   </si>
   <si>
@@ -117,6 +114,24 @@
   </si>
   <si>
     <t>Developed a Microsoft Teams notification system that posts updates to a Teams channel, tagging relevant users when tickets are updated upon workflow completion. Currently implemented for onboarding and offboarding processes, with flexibility to be reused as a sub-workflow or completion handler for future automations.</t>
+  </si>
+  <si>
+    <t>Smart Asset Billing Audit</t>
+  </si>
+  <si>
+    <t>Automates post-ticket validation in HaloPSA by analyzing closed Incident and Service Request tickets with AI to identify unbilled assets, and sends email alerts to Jason and Ashley when discrepancies are detected.</t>
+  </si>
+  <si>
+    <t>AI First Response to HaloPSA tickets</t>
+  </si>
+  <si>
+    <t>MS365, OpenAI, HaloPSA, Rewst</t>
+  </si>
+  <si>
+    <t>OpenAI, HaloPSA, MS365, Rewst</t>
+  </si>
+  <si>
+    <t>Builds an automation that sends immediate acknowledgements for new email-generated tickets, including the ticket ID to improve user communication and ensure SLA compliance, with future plans to add Microsoft Teams notifications.</t>
   </si>
 </sst>
 </file>
@@ -165,13 +180,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -507,7 +525,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D3FE286-6749-4234-BE82-DEFA19428F78}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27" style="2" bestFit="1" customWidth="1"/>
@@ -539,7 +557,7 @@
         <v>5</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>6</v>
@@ -553,7 +571,7 @@
         <v>8</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>9</v>
@@ -567,7 +585,7 @@
         <v>11</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>6</v>
@@ -581,7 +599,7 @@
         <v>15</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>6</v>
@@ -592,10 +610,10 @@
         <v>13</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>6</v>
@@ -606,10 +624,10 @@
         <v>14</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>18</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>19</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>6</v>
@@ -617,16 +635,44 @@
     </row>
     <row r="8" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>26</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -639,6 +685,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010037CFE03F1E3D084DA4C7DCDB2F33373B" ma:contentTypeVersion="5" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="48fbfec5ba6da941d58a6bba8473d12a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="9cb81d7b-fefe-42a9-a0f2-5871603dfeb9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0e0a672e89e325df77fa989dac01fde5" ns3:_="">
     <xsd:import namespace="9cb81d7b-fefe-42a9-a0f2-5871603dfeb9"/>
@@ -788,15 +843,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -806,6 +852,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8188391C-85BF-4856-861E-1F470AB9C963}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B78AE0C9-394B-4984-AE8D-B785F12488C7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -823,14 +877,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8188391C-85BF-4856-861E-1F470AB9C963}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F975563D-C219-4A29-B1CB-37D50519E395}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
updated excel for 04/29/2026
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://continuousnet-my.sharepoint.com/personal/satyam_continuous_net/Documents/Desktop/Project Tracker Dashboard/project-dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="13_ncr:1_{C4665E14-9296-465B-A7EF-B8144438D411}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E801EA7F-8186-4A6D-8878-10ED36AC1666}"/>
+  <xr:revisionPtr revIDLastSave="37" documentId="13_ncr:1_{C4665E14-9296-465B-A7EF-B8144438D411}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E4A66F11-1071-4CDF-A318-6D7F1D90D9F3}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B5181292-B819-4253-93D6-A2C77ED0862A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="38">
   <si>
     <t xml:space="preserve">Project Name </t>
   </si>
@@ -132,6 +132,24 @@
   </si>
   <si>
     <t>Builds an automation that sends immediate acknowledgements for new email-generated tickets, including the ticket ID to improve user communication and ensure SLA compliance, with future plans to add Microsoft Teams notifications.</t>
+  </si>
+  <si>
+    <t>AI Voice Agent</t>
+  </si>
+  <si>
+    <t>MS365, OpenAI, HaloPSA, Twilio</t>
+  </si>
+  <si>
+    <t>Client Face Dashboard</t>
+  </si>
+  <si>
+    <t>MS365, Ninja RMM, HaloPSA, Rewst</t>
+  </si>
+  <si>
+    <t>This project focuses on developing a dashboard that can be used by multiple clients to visualize key data. It will display insights from surveys and CSAT scores, along with service-related information such as ticket status (open, closed, categorized) and device health metrics. The dashboard will also track total workstations and patch compliance, with the ability to filter data by location and other relevant parameters.</t>
+  </si>
+  <si>
+    <t>This project involves developing a voice agent that operates after business hours to handle user calls. The agent will receive incoming calls, understand and capture the user’s issue, and either route the call to an available on-call engineer or schedule a callback if no engineer is available at that time.</t>
   </si>
 </sst>
 </file>
@@ -525,7 +543,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D3FE286-6749-4234-BE82-DEFA19428F78}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27" style="2" bestFit="1" customWidth="1"/>
@@ -672,6 +690,34 @@
         <v>31</v>
       </c>
       <c r="D10" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -685,12 +731,11 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="9cb81d7b-fefe-42a9-a0f2-5871603dfeb9" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -844,17 +889,26 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="9cb81d7b-fefe-42a9-a0f2-5871603dfeb9" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8188391C-85BF-4856-861E-1F470AB9C963}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F975563D-C219-4A29-B1CB-37D50519E395}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="9cb81d7b-fefe-42a9-a0f2-5871603dfeb9"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -878,17 +932,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F975563D-C219-4A29-B1CB-37D50519E395}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8188391C-85BF-4856-861E-1F470AB9C963}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="9cb81d7b-fefe-42a9-a0f2-5871603dfeb9"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>